<commit_message>
Revisão dos dados das Tabelas 8, 9 e 10
</commit_message>
<xml_diff>
--- a/Model Performance Metrics.xlsx
+++ b/Model Performance Metrics.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="1003" documentId="8_{EA554F94-C910-4497-9CAF-A5210DE552F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D04262D2-FADC-4D92-8608-EF3BBB76AD0E}"/>
+  <xr:revisionPtr revIDLastSave="1025" documentId="8_{EA554F94-C910-4497-9CAF-A5210DE552F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17AA27C2-C248-4381-9E3A-BE05199E5C4C}"/>
   <bookViews>
-    <workbookView xWindow="45" yWindow="1155" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{E46EFA42-E6A0-4C04-9561-DE1B488BC017}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E46EFA42-E6A0-4C04-9561-DE1B488BC017}"/>
   </bookViews>
   <sheets>
     <sheet name="In-person Environment" sheetId="5" r:id="rId1"/>
@@ -153,9 +153,6 @@
     <t>In-person and online</t>
   </si>
   <si>
-    <t>KG-BERT</t>
-  </si>
-  <si>
     <t>Guanin-Fajardo2024</t>
   </si>
   <si>
@@ -562,6 +559,9 @@
   </si>
   <si>
     <t>DOI</t>
+  </si>
+  <si>
+    <t>BiGRU + 1D-CNN</t>
   </si>
 </sst>
 </file>
@@ -620,10 +620,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -948,7 +944,7 @@
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -960,10 +956,10 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G2" t="s">
         <v>166</v>
-      </c>
-      <c r="G2" t="s">
-        <v>167</v>
       </c>
       <c r="H2" t="s">
         <v>0</v>
@@ -981,7 +977,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
@@ -1056,7 +1052,7 @@
         <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G5" t="s">
         <v>21</v>
@@ -1090,7 +1086,7 @@
         <v>20</v>
       </c>
       <c r="F6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G6" t="s">
         <v>21</v>
@@ -1128,7 +1124,7 @@
         <v>25</v>
       </c>
       <c r="F7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G7" t="s">
         <v>21</v>
@@ -1156,7 +1152,7 @@
         <v>28</v>
       </c>
       <c r="F8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G8" t="s">
         <v>21</v>
@@ -1172,19 +1168,19 @@
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" s="1">
         <v>5.25</v>
       </c>
       <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" t="s">
         <v>35</v>
-      </c>
-      <c r="F9" t="s">
-        <v>36</v>
       </c>
       <c r="G9" t="s">
         <v>21</v>
@@ -1210,19 +1206,19 @@
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D10" s="1">
         <v>4.25</v>
       </c>
       <c r="E10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" t="s">
         <v>35</v>
-      </c>
-      <c r="F10" t="s">
-        <v>36</v>
       </c>
       <c r="G10" t="s">
         <v>21</v>
@@ -1238,16 +1234,16 @@
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
         <v>39</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
       </c>
       <c r="D11" s="1">
         <v>4</v>
       </c>
       <c r="E11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1266,19 +1262,19 @@
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" s="1">
         <v>3.75</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G12" t="s">
         <v>21</v>
@@ -1302,16 +1298,16 @@
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D13" s="1">
         <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1336,16 +1332,16 @@
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D14" s="1">
         <v>5</v>
       </c>
       <c r="E14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F14" t="s">
         <v>6</v>
@@ -1370,19 +1366,19 @@
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D15" s="1">
         <v>5.5</v>
       </c>
       <c r="E15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G15" t="s">
         <v>21</v>
@@ -1402,16 +1398,16 @@
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D16" s="1">
         <v>4.25</v>
       </c>
       <c r="E16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F16" t="s">
         <v>14</v>
@@ -1430,19 +1426,19 @@
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D17" s="1">
         <v>5.5</v>
       </c>
       <c r="E17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G17" t="s">
         <v>21</v>
@@ -1462,10 +1458,10 @@
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" s="1">
         <v>4.25</v>
@@ -1474,7 +1470,7 @@
         <v>20</v>
       </c>
       <c r="F18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G18" t="s">
         <v>21</v>
@@ -1498,19 +1494,19 @@
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D19" s="1">
         <v>5.5</v>
       </c>
       <c r="E19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F19" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G19" t="s">
         <v>21</v>
@@ -1534,16 +1530,16 @@
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
+        <v>129</v>
+      </c>
+      <c r="C20" t="s">
         <v>130</v>
-      </c>
-      <c r="C20" t="s">
-        <v>131</v>
       </c>
       <c r="D20" s="1">
         <v>5</v>
       </c>
       <c r="E20" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F20" t="s">
         <v>6</v>
@@ -1572,19 +1568,19 @@
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C21" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D21" s="1">
         <v>5</v>
       </c>
       <c r="E21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F21" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G21" t="s">
         <v>21</v>
@@ -1610,19 +1606,19 @@
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C22" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D22" s="1">
         <v>4.5</v>
       </c>
       <c r="E22" t="s">
+        <v>34</v>
+      </c>
+      <c r="F22" t="s">
         <v>35</v>
-      </c>
-      <c r="F22" t="s">
-        <v>36</v>
       </c>
       <c r="G22" t="s">
         <v>21</v>
@@ -1640,19 +1636,19 @@
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
+        <v>145</v>
+      </c>
+      <c r="C23" t="s">
         <v>146</v>
-      </c>
-      <c r="C23" t="s">
-        <v>147</v>
       </c>
       <c r="D23" s="1">
         <v>5</v>
       </c>
       <c r="E23" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G23" t="s">
         <v>21</v>
@@ -1666,19 +1662,19 @@
     </row>
     <row r="24" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C24" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D24" s="1">
         <v>5</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F24" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G24" t="s">
         <v>21</v>
@@ -1702,19 +1698,19 @@
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D25" s="1">
         <v>4.5</v>
       </c>
       <c r="E25" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G25" t="s">
         <v>21</v>
@@ -1736,19 +1732,19 @@
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D26" s="1">
         <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F26" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G26" t="s">
         <v>21</v>
@@ -2693,7 +2689,7 @@
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -2705,10 +2701,10 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G2" t="s">
         <v>166</v>
-      </c>
-      <c r="G2" t="s">
-        <v>167</v>
       </c>
       <c r="H2" t="s">
         <v>0</v>
@@ -2726,7 +2722,7 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
@@ -2740,7 +2736,7 @@
         <v>5.5</v>
       </c>
       <c r="E3" t="s">
-        <v>32</v>
+        <v>168</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
@@ -2765,10 +2761,10 @@
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D4" s="1">
         <v>3.75</v>
@@ -2777,7 +2773,7 @@
         <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G4" t="s">
         <v>31</v>
@@ -2796,24 +2792,24 @@
       </c>
       <c r="L4" s="3"/>
       <c r="M4" s="2">
-        <v>6479</v>
+        <v>589</v>
       </c>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D5" s="1">
         <v>3.75</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G5" t="s">
         <v>31</v>
@@ -2831,19 +2827,19 @@
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D6" s="1">
         <v>4</v>
       </c>
       <c r="E6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G6" t="s">
         <v>31</v>
@@ -2867,19 +2863,19 @@
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D7" s="1">
         <v>5</v>
       </c>
       <c r="E7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G7" t="s">
         <v>31</v>
@@ -2903,19 +2899,19 @@
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D8" s="1">
         <v>6</v>
       </c>
       <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
         <v>35</v>
-      </c>
-      <c r="F8" t="s">
-        <v>36</v>
       </c>
       <c r="G8" t="s">
         <v>31</v>
@@ -2929,19 +2925,19 @@
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D9" s="1">
         <v>6</v>
       </c>
       <c r="E9" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" t="s">
         <v>35</v>
-      </c>
-      <c r="F9" t="s">
-        <v>36</v>
       </c>
       <c r="G9" t="s">
         <v>31</v>
@@ -2959,19 +2955,19 @@
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D10" s="1">
         <v>3.75</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F10" t="s">
-        <v>6</v>
+        <v>124</v>
       </c>
       <c r="G10" t="s">
         <v>31</v>
@@ -2993,19 +2989,19 @@
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
+        <v>125</v>
+      </c>
+      <c r="C11" t="s">
         <v>126</v>
-      </c>
-      <c r="C11" t="s">
-        <v>127</v>
       </c>
       <c r="D11" s="1">
         <v>4.75</v>
       </c>
       <c r="E11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G11" t="s">
         <v>31</v>
@@ -3031,19 +3027,19 @@
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D12" s="1">
         <v>4.25</v>
       </c>
       <c r="E12" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G12" t="s">
         <v>31</v>
@@ -3071,7 +3067,7 @@
         <v>5.5</v>
       </c>
       <c r="E14" t="str">
-        <v>KG-BERT</v>
+        <v>BiGRU + 1D-CNN</v>
       </c>
       <c r="F14" t="str">
         <v>Deep Learning</v>
@@ -3100,34 +3096,34 @@
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
-        <v>10.1109/IIPEM65914.2025.11548244</v>
+        <v>10.5281/zenodo.8115647</v>
       </c>
       <c r="C15" t="str">
-        <v>Khasne2025</v>
+        <v>Cohausz2023125</v>
       </c>
       <c r="D15" s="1">
-        <v>3.75</v>
+        <v>6</v>
       </c>
       <c r="E15" t="str">
-        <v>RNN-SVM</v>
+        <v>XGBoost</v>
       </c>
       <c r="F15" t="str">
-        <v>Deep Learning</v>
+        <v>Ensemble Learning</v>
       </c>
       <c r="G15" t="str">
         <v>In-person and online</v>
       </c>
       <c r="H15" s="3">
-        <v>0.97799999999999998</v>
+        <v>0</v>
       </c>
       <c r="I15" s="3">
-        <v>0.97499999999999998</v>
+        <v>0</v>
       </c>
       <c r="J15" s="3">
-        <v>0.97899999999999998</v>
+        <v>0</v>
       </c>
       <c r="K15" s="3">
-        <v>0.97699999999999998</v>
+        <v>0</v>
       </c>
       <c r="L15" s="3">
         <v>0</v>
@@ -3138,10 +3134,10 @@
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
-        <v>10.5281/zenodo.8115647</v>
+        <v>10.5281/zenodo.14503515</v>
       </c>
       <c r="C16" t="str">
-        <v>Cohausz2023125</v>
+        <v>Cohausz2024177</v>
       </c>
       <c r="D16" s="1">
         <v>6</v>
@@ -3165,27 +3161,27 @@
         <v>0</v>
       </c>
       <c r="K16" s="3">
-        <v>0</v>
+        <v>0.91</v>
       </c>
       <c r="L16" s="3">
         <v>0</v>
       </c>
       <c r="M16" s="2">
-        <v>0</v>
+        <v>22437</v>
       </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
-        <v>10.5281/zenodo.14503515</v>
+        <v>10.1016/j.eswa.2025.128724</v>
       </c>
       <c r="C17" t="str">
-        <v>Cohausz2024177</v>
+        <v>Hakkal2025</v>
       </c>
       <c r="D17" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E17" t="str">
-        <v>XGBoost</v>
+        <v>GNN + LightGBM</v>
       </c>
       <c r="F17" t="str">
         <v>Ensemble Learning</v>
@@ -3194,36 +3190,36 @@
         <v>In-person and online</v>
       </c>
       <c r="H17" s="3">
-        <v>0</v>
+        <v>0.83089999999999997</v>
       </c>
       <c r="I17" s="3">
-        <v>0</v>
+        <v>0.81100000000000005</v>
       </c>
       <c r="J17" s="3">
-        <v>0</v>
+        <v>0.93289999999999995</v>
       </c>
       <c r="K17" s="3">
-        <v>0.91</v>
+        <v>0.86770000000000003</v>
       </c>
       <c r="L17" s="3">
-        <v>0</v>
+        <v>0.91479999999999995</v>
       </c>
       <c r="M17" s="2">
-        <v>22437</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
-        <v>10.1016/j.eswa.2025.128724</v>
+        <v>10.7717/peerj-cs.3792</v>
       </c>
       <c r="C18" t="str">
-        <v>Hakkal2025</v>
+        <v>Taqatqeh2026</v>
       </c>
       <c r="D18" s="1">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="E18" t="str">
-        <v>GNN + LightGBM</v>
+        <v>Boosting + GridSearch</v>
       </c>
       <c r="F18" t="str">
         <v>Ensemble Learning</v>
@@ -3232,74 +3228,74 @@
         <v>In-person and online</v>
       </c>
       <c r="H18" s="3">
-        <v>0.83089999999999997</v>
+        <v>0.89700000000000002</v>
       </c>
       <c r="I18" s="3">
-        <v>0.81100000000000005</v>
+        <v>0.88</v>
       </c>
       <c r="J18" s="3">
-        <v>0.93289999999999995</v>
+        <v>0.92</v>
       </c>
       <c r="K18" s="3">
-        <v>0.86770000000000003</v>
+        <v>0.9</v>
       </c>
       <c r="L18" s="3">
-        <v>0.91479999999999995</v>
+        <v>0.92</v>
       </c>
       <c r="M18" s="2">
-        <v>0</v>
+        <v>2120</v>
       </c>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" t="str">
-        <v>10.7717/peerj-cs.3792</v>
+        <v>10.1109/IEHNS68708.2026.11606961</v>
       </c>
       <c r="C19" t="str">
-        <v>Taqatqeh2026</v>
+        <v>Xiao2026</v>
       </c>
       <c r="D19" s="1">
-        <v>4.75</v>
+        <v>4.25</v>
       </c>
       <c r="E19" t="str">
-        <v>Boosting + GridSearch</v>
+        <v>Optimized Fusion Model</v>
       </c>
       <c r="F19" t="str">
-        <v>Ensemble Learning</v>
+        <v>Machine Learning</v>
       </c>
       <c r="G19" t="str">
         <v>In-person and online</v>
       </c>
       <c r="H19" s="3">
-        <v>0.89700000000000002</v>
+        <v>0.93500000000000005</v>
       </c>
       <c r="I19" s="3">
-        <v>0.88</v>
+        <v>0</v>
       </c>
       <c r="J19" s="3">
-        <v>0.92</v>
+        <v>0</v>
       </c>
       <c r="K19" s="3">
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="L19" s="3">
-        <v>0.92</v>
+        <v>0</v>
       </c>
       <c r="M19" s="2">
-        <v>2120</v>
+        <v>400</v>
       </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B20" t="str">
-        <v>10.1109/IEHNS68708.2026.11606961</v>
+        <v>10.1109/ACCESS.2022.3195531</v>
       </c>
       <c r="C20" t="str">
-        <v>Xiao2026</v>
+        <v>Czibula202280651</v>
       </c>
       <c r="D20" s="1">
-        <v>4.25</v>
+        <v>4</v>
       </c>
       <c r="E20" t="str">
-        <v>Optimized Fusion Model</v>
+        <v>Polynomial Regression</v>
       </c>
       <c r="F20" t="str">
         <v>Machine Learning</v>
@@ -3308,36 +3304,36 @@
         <v>In-person and online</v>
       </c>
       <c r="H20" s="3">
-        <v>0.93500000000000005</v>
+        <v>0.92920000000000003</v>
       </c>
       <c r="I20" s="3">
-        <v>0</v>
+        <v>0.95650000000000002</v>
       </c>
       <c r="J20" s="3">
-        <v>0</v>
+        <v>0.92920000000000003</v>
       </c>
       <c r="K20" s="3">
-        <v>0</v>
+        <v>0.93799999999999994</v>
       </c>
       <c r="L20" s="3">
         <v>0</v>
       </c>
       <c r="M20" s="2">
-        <v>400</v>
+        <v>506</v>
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
-        <v>10.1109/ACCESS.2022.3195531</v>
+        <v>10.1109/FIE63693.2025.11328252</v>
       </c>
       <c r="C21" t="str">
-        <v>Czibula202280651</v>
+        <v>Abdelhamid2025</v>
       </c>
       <c r="D21" s="1">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="E21" t="str">
-        <v>Polynomial Regression</v>
+        <v>Logistic Regression</v>
       </c>
       <c r="F21" t="str">
         <v>Machine Learning</v>
@@ -3346,36 +3342,36 @@
         <v>In-person and online</v>
       </c>
       <c r="H21" s="3">
-        <v>0.92920000000000003</v>
+        <v>0.95989999999999998</v>
       </c>
       <c r="I21" s="3">
-        <v>0.95650000000000002</v>
+        <v>0.96750000000000003</v>
       </c>
       <c r="J21" s="3">
-        <v>0.92920000000000003</v>
+        <v>0.95269999999999999</v>
       </c>
       <c r="K21" s="3">
-        <v>0.93799999999999994</v>
+        <v>0.96009999999999995</v>
       </c>
       <c r="L21" s="3">
         <v>0</v>
       </c>
       <c r="M21" s="2">
-        <v>506</v>
+        <v>589</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" t="str">
-        <v>10.1109/FIE63693.2025.11328252</v>
+        <v>10.1007/s42979-022-01251-5</v>
       </c>
       <c r="C22" t="str">
-        <v>Abdelhamid2025</v>
+        <v>Dang2022</v>
       </c>
       <c r="D22" s="1">
         <v>3.75</v>
       </c>
       <c r="E22" t="str">
-        <v>Logistic Regression</v>
+        <v>Decision Tree</v>
       </c>
       <c r="F22" t="str">
         <v>Machine Learning</v>
@@ -3384,36 +3380,36 @@
         <v>In-person and online</v>
       </c>
       <c r="H22" s="3">
-        <v>0.95989999999999998</v>
+        <v>0.47199999999999998</v>
       </c>
       <c r="I22" s="3">
-        <v>0.96750000000000003</v>
+        <v>0</v>
       </c>
       <c r="J22" s="3">
-        <v>0.95269999999999999</v>
+        <v>0</v>
       </c>
       <c r="K22" s="3">
-        <v>0.96009999999999995</v>
+        <v>0</v>
       </c>
       <c r="L22" s="3">
         <v>0</v>
       </c>
       <c r="M22" s="2">
-        <v>6479</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B23" t="str">
-        <v>10.1007/s42979-022-01251-5</v>
+        <v>10.1109/IIPEM65914.2025.11548244</v>
       </c>
       <c r="C23" t="str">
-        <v>Dang2022</v>
+        <v>Khasne2025</v>
       </c>
       <c r="D23" s="1">
         <v>3.75</v>
       </c>
       <c r="E23" t="str">
-        <v>Decision Tree</v>
+        <v>RNN-SVM</v>
       </c>
       <c r="F23" t="str">
         <v>Machine Learning</v>
@@ -3422,22 +3418,22 @@
         <v>In-person and online</v>
       </c>
       <c r="H23" s="3">
-        <v>0.47199999999999998</v>
+        <v>0.97799999999999998</v>
       </c>
       <c r="I23" s="3">
-        <v>0</v>
+        <v>0.97499999999999998</v>
       </c>
       <c r="J23" s="3">
-        <v>0</v>
+        <v>0.97899999999999998</v>
       </c>
       <c r="K23" s="3">
-        <v>0</v>
+        <v>0.97699999999999998</v>
       </c>
       <c r="L23" s="3">
         <v>0</v>
       </c>
       <c r="M23" s="2">
-        <v>326</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3453,7 +3449,7 @@
   <sheetData>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -3465,10 +3461,10 @@
         <v>7</v>
       </c>
       <c r="F2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G2" t="s">
         <v>166</v>
-      </c>
-      <c r="G2" t="s">
-        <v>167</v>
       </c>
       <c r="H2" t="s">
         <v>0</v>
@@ -3486,27 +3482,27 @@
         <v>4</v>
       </c>
       <c r="M2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D3" s="1">
         <v>3.75</v>
       </c>
       <c r="E3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G3" t="s">
         <v>82</v>
-      </c>
-      <c r="F3" t="s">
-        <v>125</v>
-      </c>
-      <c r="G3" t="s">
-        <v>83</v>
       </c>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
@@ -3519,22 +3515,22 @@
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D4" s="1">
         <v>4</v>
       </c>
       <c r="E4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H4" s="3">
         <v>0.72560000000000002</v>
@@ -3549,22 +3545,22 @@
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D5" s="1">
         <v>4.25</v>
       </c>
       <c r="E5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
       </c>
       <c r="G5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H5" s="3">
         <v>0.95099999999999996</v>
@@ -3581,22 +3577,22 @@
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D6" s="1">
         <v>4.5</v>
       </c>
       <c r="E6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
       </c>
       <c r="G6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H6" s="3">
         <v>0.86799999999999999</v>
@@ -3615,22 +3611,22 @@
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D7" s="1">
         <v>3.75</v>
       </c>
       <c r="E7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
       </c>
       <c r="G7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H7" s="3">
         <v>0.95199999999999996</v>
@@ -3649,22 +3645,22 @@
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D8" s="1">
         <v>4</v>
       </c>
       <c r="E8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H8" s="3">
         <v>0.96</v>
@@ -3685,22 +3681,22 @@
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D9" s="1">
         <v>3.75</v>
       </c>
       <c r="E9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
       </c>
       <c r="G9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H9" s="3">
         <v>0.83</v>
@@ -3715,22 +3711,22 @@
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D10" s="1">
         <v>4.75</v>
       </c>
       <c r="E10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
       </c>
       <c r="G10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H10" s="3">
         <v>0.90129999999999999</v>
@@ -3753,22 +3749,22 @@
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D11" s="1">
         <v>5</v>
       </c>
       <c r="E11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
       </c>
       <c r="G11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H11" s="3">
         <v>0.98499999999999999</v>
@@ -3789,22 +3785,22 @@
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D12" s="1">
         <v>4.5</v>
       </c>
       <c r="E12" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H12" s="3">
         <v>0.87</v>
@@ -3825,22 +3821,22 @@
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D13" s="1">
         <v>5.5</v>
       </c>
       <c r="E13" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H13" s="3">
         <v>0.79449999999999998</v>
@@ -3855,22 +3851,22 @@
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C14" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D14" s="1">
         <v>5.25</v>
       </c>
       <c r="E14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F14" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H14" s="3">
         <v>0.87</v>
@@ -3889,22 +3885,22 @@
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D15" s="1">
         <v>3.75</v>
       </c>
       <c r="E15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F15" t="s">
         <v>6</v>
       </c>
       <c r="G15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H15" s="3">
         <v>0.97199999999999998</v>
@@ -3923,22 +3919,22 @@
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D16" s="1">
         <v>4</v>
       </c>
       <c r="E16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H16" s="3">
         <v>0.97099999999999997</v>
@@ -3953,22 +3949,22 @@
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D17" s="1">
         <v>4.75</v>
       </c>
       <c r="E17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F17" t="s">
         <v>6</v>
       </c>
       <c r="G17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
@@ -3985,22 +3981,22 @@
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
+        <v>140</v>
+      </c>
+      <c r="C18" t="s">
         <v>141</v>
-      </c>
-      <c r="C18" t="s">
-        <v>142</v>
       </c>
       <c r="D18" s="1">
         <v>5.5</v>
       </c>
       <c r="E18" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H18" s="3">
         <v>0.92</v>
@@ -4019,22 +4015,22 @@
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
+        <v>150</v>
+      </c>
+      <c r="C19" t="s">
         <v>151</v>
-      </c>
-      <c r="C19" t="s">
-        <v>152</v>
       </c>
       <c r="D19" s="1">
         <v>5</v>
       </c>
       <c r="E19" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F19" t="s">
         <v>6</v>
       </c>
       <c r="G19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H19" s="3">
         <v>0.92400000000000004</v>
@@ -4057,22 +4053,22 @@
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C20" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D20" s="1">
         <v>4</v>
       </c>
       <c r="E20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H20" s="3">
         <v>0.66</v>
@@ -4095,22 +4091,22 @@
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D21" s="1">
         <v>4.75</v>
       </c>
       <c r="E21" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F21" t="s">
         <v>6</v>
       </c>
       <c r="G21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H21" s="3">
         <v>0.92400000000000004</v>
@@ -4318,7 +4314,7 @@
       <c r="L27" s="3">
         <v>0.94599999999999995</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27">
         <v>32593</v>
       </c>
     </row>

</xml_diff>